<commit_message>
Add 2025-26 top scorers and scraping updates
</commit_message>
<xml_diff>
--- a/ligat_haal_project/notebooks/attendance/ligat_haal_2024_2025_attendance.xlsx
+++ b/ligat_haal_project/notebooks/attendance/ligat_haal_2024_2025_attendance.xlsx
@@ -319,7 +319,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -383,10 +383,10 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">

</xml_diff>